<commit_message>
chore: update ETRA-Riyadh-Sales-August-Example.xlsx with revised data for improved accuracy and presentation quality
</commit_message>
<xml_diff>
--- a/web-presentation/pdf-exports/ETRA-Riyadh-Sales-August-Example.xlsx
+++ b/web-presentation/pdf-exports/ETRA-Riyadh-Sales-August-Example.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص_أغسطس" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حسب_المنتج" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حسب_الأسبوع" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حسب_القطاع" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="أوامر_للتجربة" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تمارين_عملية_وأوامر" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص_أغسطس" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حسب_المنتج" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حسب_الأسبوع" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حسب_القطاع" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="أوامر_للتجربة" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +75,18 @@
       <b val="1"/>
       <color rgb="002E7D32"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B71C1C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="7">
@@ -135,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -157,6 +170,20 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -522,6 +549,399 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="95" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>تمارين عملية + أوامر جاهزة للورشة (يوم 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ارفع ملف مبيعات الرياض مع التمارين التي تحتاج بيانات. انسخ الأمر من عمود «نص الأمر».</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>رقم</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>التمرين</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>وصف سريع</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>نص الأمر (انسخه)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="74" customHeight="1">
+      <c r="A5" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>أمر سيء → أمر قوي</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>ابنِ الأمر الضعيف إلى أمر كامل العناصر قدام القاعة</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>هذا أمر ضعيف: «لخّص لي الملف».
+أعد كتابته كأمر احترافي كامل العناصر:
+السياق + الدور + الجمهور + الشكل + القيود + المهمة.
+استخدم ملف مبيعات فرع الرياض (هدف 1,200,000 / متحقق 980,000) إن لزم.
+لا تخترع أرقامًا غير موجودة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="74" customHeight="1">
+      <c r="A6" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>نفس المهمة… دوران (أ) محلل</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>شغّل هذا الأمر أولًا على ملف الرياض</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>الدور: أنت محلل إداري محترف.
+الجمهور: المدير التنفيذي.
+الشكل: 5 نقاط + توصية واحدة.
+القيود: لا تخترع أرقامًا؛ اللهجة رسمية قصيرة.
+المهمة: حلّل فجوة مبيعات فرع الرياض في أغسطس من الملف المرفق.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="74" customHeight="1">
+      <c r="A7" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>نفس المهمة… دوران (ب) كاتب إعلانات</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>شغّل هذا الأمر ثانيًا وقارن النبرة</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>الدور: أنت كاتب إعلانات تسويقية.
+الجمهور: عملاء على لينكدإن.
+الشكل: منشور قصير (خطاف + فائدة + سؤال).
+القيود: ممنوع ذكر أرقام داخلية أو أسماء فروع سرية؛ اللهجة ودّية مهنية.
+المهمة: استخرج رسالة عامة من نفس ملف المبيعات بدون كشف بيانات حسّاسة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="116" customHeight="1">
+      <c r="A8" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>نفس الحقيقة… 3 جماهير</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>مدير / فريق / لينكدإن من نفس الرقم</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>الحقيقة الثابتة: مبيعات فرع الرياض في أغسطس 980,000 من أصل هدف 1,200,000 (فجوة 220,000).
+اكتب 3 نسخ:
+1) للمدير التنفيذي (مختصر + قرار مطلوب)
+2) لفريق المبيعات (تفاصيل تنفيذ)
+3) لمنشور لينكدإن عام (بدون أرقام داخلية)
+قيود: لا تخترع أسبابًا غير موجودة؛ إن احتجت سببًا غير متوفر اكتب «غير متوفر».</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="214" customHeight="1">
+      <c r="A9" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Few-Shot إيميل دعم</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>مثالين ثم مهمة جديدة بنفس الأسلوب</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>قلّد نفس أسلوب الإيميلين التاليين حرفيًا في النبرة والطول والهيكل.
+مثال 1:
+المدخل: عميل يقول تأخر الطلب رقم 4412 يومين.
+المخرج: موضوع: تحديث طلبك 4412
+مرحباً أحمد، نعتذر عن التأخر. طلبك 4412 في مرحلة الشحن ويصل خلال 24–48 ساعة. إذا احتجت مساعدة إضافية رد على هذا الإيميل. شكرًا لتفهمك.
+مثال 2:
+المدخل: عميلة تسأل عن استبدال سماعة تالفة.
+المخرج: موضوع: طلب استبدال سماعة
+مرحباً سارة، يمكننا استبدال السماعة خلال 7 أيام من الاستلام. أرسلي صورة للعيب ورقم الطلب وسنجهّز بوليصة الإرجاع خلال يوم عمل. شكرًا لتواصلك.
+المهمة الآن:
+المدخل: عميل يقول إن الفاتورة وصلت بمبلغ أعلى من المتفق.
+اكتب إيميل بنفس الأسلوب تمامًا.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>هلوسة — بدون قيد</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>اعرض الناتج الأول للقاعة</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>كم كان عدد موظفي أرامكو في سنة 2018 بالضبط؟ أعطني رقمًا واحدًا فقط.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>هلوسة — مع قيد لا أعرف</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>قارن مع الأمر السابق</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>كم كان عدد موظفي أرامكو في سنة 2018 بالضبط؟
+إن لم يكن لديك مصدر موثوق مؤكد اكتب فقط: لا أعرف.
+لا تخمّن ولا تختلق رقمًا.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="130" customHeight="1">
+      <c r="A12" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>المسار الكامل PDF→إيميل→تغريدات</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>تمرين المساعد الإداري الذكي</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>ارفع/استخدم ملف مبيعات الرياض المرفق ونفّذ بالترتيب دون اختراع أرقام:
+الخطوة 1: لخّص للإدارة في 5 نقاط مرقّمة + توصية واحدة.
+الخطوة 2: حوّل نقاط الخطوة 1 فقط إلى إيميل رسمي للمدير التنفيذي
+(غرض في سطر + 3 نقاط + طلب إجراء واحد + خاتمة).
+الخطوة 3: اكتب 3 تغريدات/منشورات قصيرة لجمهور عام
+(خطاف + فائدة + سؤال) بدون أرقام أو أسماء داخلية حسّاسة.
+الخطوة 4: في نهاية ردك ضع قائمة تحقق نعم/لا:
+الأرقام مطابقة؟ الأسماء صحيحة؟ طلب إجراء واحد؟ المنشورات آمنة؟</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="116" customHeight="1">
+      <c r="A13" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>فصل حقيقة / رأي / غير مؤكد</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Checklist جودة البحث</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>هذا ملخص:
+«مبيعات الرياض 980 ألف من هدف 1.2 مليون. لذلك يجب زيادة ميزانية الإعلانات 25% فورًا لأن المنافس سيطر على السوق بالكامل، ومتوقع أن ترتفع المبيعات 40% الشهر القادم.»
+صنّف كل جملة إلى: حقيقة من الملف | رأي/توصية | غير مؤكد/مختلق.
+بعدها أعد كتابة الملخص بحيث:
+- الحقائق فقط أولًا
+- التوصيات منفصلة
+- أي شيء غير مدعوم يُوسم: غير مؤكد</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="88" customHeight="1">
+      <c r="A14" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>طقم طوارئ — مهمة حقيقية</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>يملأ الطالب الحقول بين الأقواس</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>السياق: [صف مهمتك الحقيقية + أي ملف/نقاط]
+الدور: أنت [محلل/محرر/مسؤول دعم] بخبرة في [المجال]
+الجمهور: [مدير / فريق / عملاء]
+الشكل: [إيميل / 5 نقاط / جدول / منشور]
+القيود: الطول [X]؛ اللهجة [رسمية قصيرة]؛ لا تخترع أرقامًا؛ قل لا أعرف إن لم تكن متأكدًا
+المهمة: [اكتب المطلوب النهائي بجملة واضحة]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="144" customHeight="1">
+      <c r="A15" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>تشخيص أخطاء الأمر (1–5)</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>لعبة سريعة مع القاعة</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>هذا أمر:
+«اكتب لي بسرعة شيء حلو عن المبيعات للجميع وبشكل جيد وطويل ومختصر بنفس الوقت.»
+1) ما أرقام الأخطاء الموجودة من قائمة الورشة؟
+   1 غامض بلا هدف
+   2 بلا جمهور/رسمية
+   3 بلا شكل مخرجات
+   4 قبول بلا تحقق (إن ظهر)
+   5 طويل بلا أولوية
+2) أعد كتابة الأمر صحيحًا بالعناصر الستة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>مقارنة أساسية — أمر ضعيف</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>من ورقة أوامر_للتجربة الأصلية</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>اكتب لي عن التقرير.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="220" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>مقارنة أساسية — أمر قوي</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>مع رفع ملف الرياض</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>السياق: هذا ملف مبيعات فرع الرياض لشهر أغسطس 2025. الهدف 1,200,000 ريال والمتحقق 980,000 ريال. ركّز على أسباب الفجوة لا على الإنجازات العامة.
+الدور: أنت محلل إداري محترف في مبيعات التجزئة والتقنية.
+الجمهور: المدير التنفيذي مشغول ويحتاج قرار سريع.
+الشكل:
+1) ملخص تنفيذي في 4 أسطر كحد أقصى
+2) 5 نقاط مرقّمة لأهم أسباب الفجوة مع ربطها بأرقام من الملف فقط
+3) جدول صغير: السبب | الأثر التقريبي | دليل من الملف
+4) توصية واحدة واضحة للأسبوع القادم في سطرين
+القيود:
+- لا تخترع أرقامًا غير موجودة في الملف
+- إن نقص رقم أو معلومة اكتب: غير متوفر في الملف
+- اللهجة رسمية قصيرة
+- افصل الحقائق عن رأيك
+المهمة: حلّل الملف واستخرج أسباب فجوة مبيعات أغسطس في فرع الرياض مع توصية تنفيذية واحدة.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -698,7 +1118,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -893,7 +1313,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1007,7 +1427,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1112,49 +1532,48 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>أمران جاهزان للتجربة مع الذكاء الاصطناعي</t>
+          <t>أمران أساسيان للمقارنة السريعة</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>الأمر 1 — ضعيف (للمقارنة)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>الأمر 1 — ضعيف</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>اكتب لي عن التقرير.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>الأمر 2 — قوي (انسخه مع الملف)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="220" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>الأمر 2 — قوي</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="210" customHeight="1">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>السياق: هذا ملف مبيعات فرع الرياض لشهر أغسطس 2025. الهدف 1,200,000 ريال والمتحقق 980,000 ريال. ركّز على أسباب الفجوة لا على الإنجازات العامة.
 الدور: أنت محلل إداري محترف في مبيعات التجزئة والتقنية.
@@ -1173,27 +1592,8 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>طريقة التجربة</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="80" customHeight="1">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>1) ارفع هذا الملف على ChatGPT أو Claude أو Gemini
-2) الصق الأمر الضعيف أولًا ولاحظ الناتج
-3) الصق الأمر القوي على نفس الملف وقارن الوضوح والدقة
-4) راجع الأرقام يدويًا مع ورقة ملخص_أغسطس</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A10:B10"/>
+  <mergeCells count="2">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A7:B7"/>
   </mergeCells>

</xml_diff>